<commit_message>
Nov Release done and preparing for execution
</commit_message>
<xml_diff>
--- a/Encollect_Web_SCB_P3/Cypress/fixtures/ProductMasterTemplate.xlsx
+++ b/Encollect_Web_SCB_P3/Cypress/fixtures/ProductMasterTemplate.xlsx
@@ -401,112 +401,112 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kids</v>
+        <v>Movies</v>
       </c>
       <c r="B2" t="str">
-        <v>Incredible Bamboo Towels</v>
+        <v>Practical Rubber Salad</v>
       </c>
       <c r="C2" t="str">
-        <v>Intelligent</v>
+        <v>Practical</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Books</v>
+        <v>Grocery</v>
       </c>
       <c r="B3" t="str">
-        <v>Handcrafted Marble Tuna</v>
+        <v>Modern Silk Salad</v>
       </c>
       <c r="C3" t="str">
-        <v>Bespoke</v>
+        <v>Awesome</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Tools</v>
+        <v>Toys</v>
       </c>
       <c r="B4" t="str">
-        <v>Sleek Bronze Sausages</v>
+        <v>Elegant Rubber Keyboard</v>
       </c>
       <c r="C4" t="str">
-        <v>Ergonomic</v>
+        <v>Fantastic</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Toys</v>
+        <v>Beauty</v>
       </c>
       <c r="B5" t="str">
-        <v>Incredible Bronze Chips</v>
+        <v>Sleek Ceramic Tuna</v>
       </c>
       <c r="C5" t="str">
-        <v>Unbranded</v>
+        <v>Bespoke</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Games</v>
+        <v>Beauty</v>
       </c>
       <c r="B6" t="str">
-        <v>Elegant Bamboo Table</v>
+        <v>Incredible Rubber Bike</v>
       </c>
       <c r="C6" t="str">
-        <v>Rustic</v>
+        <v>Elegant</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Books</v>
+        <v>Music</v>
       </c>
       <c r="B7" t="str">
-        <v>Licensed Plastic Mouse</v>
+        <v>Gorgeous Ceramic Cheese</v>
       </c>
       <c r="C7" t="str">
-        <v>Elegant</v>
+        <v>Unbranded</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Clothing</v>
+        <v>Automotive</v>
       </c>
       <c r="B8" t="str">
-        <v>Oriental Bronze Shoes</v>
+        <v>Awesome Bamboo Chair</v>
       </c>
       <c r="C8" t="str">
-        <v>Luxurious</v>
+        <v>Ergonomic</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Music</v>
+        <v>Electronics</v>
       </c>
       <c r="B9" t="str">
-        <v>Intelligent Ceramic Soap</v>
+        <v>Incredible Bamboo Sausages</v>
       </c>
       <c r="C9" t="str">
-        <v>Unbranded</v>
+        <v>Recycled</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Kids</v>
+        <v>Toys</v>
       </c>
       <c r="B10" t="str">
-        <v>Handmade Rubber Towels</v>
+        <v>Fantastic Marble Shirt</v>
       </c>
       <c r="C10" t="str">
-        <v>Modern</v>
+        <v>Incredible</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Toys</v>
+        <v>Outdoors</v>
       </c>
       <c r="B11" t="str">
-        <v>Intelligent Marble Pants</v>
+        <v>Electronic Ceramic Bacon</v>
       </c>
       <c r="C11" t="str">
-        <v>Small</v>
+        <v>Generic</v>
       </c>
     </row>
   </sheetData>

</xml_diff>